<commit_message>
- Suppression du SNR - SourcePatientInfo  => référence à PAM et à l'annexe INS XDM SourcePatientId => Référence à l'annexe INS et au volet partage 9cac699e80e0c45cf191134845967a57a12fbac2
</commit_message>
<xml_diff>
--- a/spec-tech/ig/StructureDefinition-xdmAuthor.xlsx
+++ b/spec-tech/ig/StructureDefinition-xdmAuthor.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-23T16:11:23+00:00</t>
+    <t>2026-07-27T13:36:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -87,7 +87,6 @@
 - Un professionnel (personne physique) via son logiciel de professionnel, 
 - Le patient/usager (personne physique) via Mon espace Santé, 
 - Un système de structure (dispositif, automate, appareil connecté…), 
-- Un SNR (Service Numérique Référencé), 
 **author** est un ensemble constitué des sous-attributs **authorInstitution** , **authorPerson**, **authorRole** et **authorSpecialty** et ne porte pas de valeur par lui-même. </t>
   </si>
   <si>
@@ -274,7 +273,7 @@
   </si>
   <si>
     <t>https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/xdmActorPs
-https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/xdmActorPatienthttps://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/xdmActorSnrhttps://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/xdmActorSystem</t>
+https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/xdmActorPatienthttps://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/xdmActorSystem</t>
   </si>
   <si>
     <t>Author</t>
@@ -623,7 +622,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="185.20703125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="125.8125" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>